<commit_message>
previous update didn't work properly, resolved now
</commit_message>
<xml_diff>
--- a/data/metabarcoding/COI/FC-COI_Metabarcoding_OBIS_sample_metadata.xlsx
+++ b/data/metabarcoding/COI/FC-COI_Metabarcoding_OBIS_sample_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matt.lemay/Dropbox/1.Hakai_Biodiversity/1.ResearchProjects/2.BioBlitzes/2022_False Creek Bioblitz/OBIS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tim.vanderstap\Desktop\GitHub\2022-FalseCreek-eDNA\data\metabarcoding\COI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3027225B-A1B7-504F-8ADE-873EF4EEC64D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE945D32-02F8-4B9D-BE70-21AA514FED6B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="500" windowWidth="48480" windowHeight="26560" activeTab="1" xr2:uid="{ADB8ACBB-6211-4A34-8A90-253E464AEC74}"/>
+    <workbookView xWindow="15" yWindow="495" windowWidth="48480" windowHeight="26565" activeTab="1" xr2:uid="{ADB8ACBB-6211-4A34-8A90-253E464AEC74}"/>
   </bookViews>
   <sheets>
     <sheet name="data-dictionary" sheetId="1" r:id="rId1"/>
@@ -564,9 +564,6 @@
     <t>Cytochrome c oxidase subunit I</t>
   </si>
   <si>
-    <t>mICOIintF</t>
-  </si>
-  <si>
     <t>dgHCO2198R</t>
   </si>
   <si>
@@ -629,6 +626,9 @@
       </rPr>
       <t> (2013) https://doi.org/10.1186/1742-9994-10-34; Meyer (2003) https://doi.org/10.1046/j.1095-8312.2003.00197.x</t>
     </r>
+  </si>
+  <si>
+    <t>mlCOIintF</t>
   </si>
 </sst>
 </file>
@@ -1072,15 +1072,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E97C17E1-FA21-4BEA-987A-AB81EBDEE92A}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="149.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="148.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="149.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="148.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1094,7 +1094,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1133,7 +1133,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1158,7 +1158,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1169,7 +1169,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1180,7 +1180,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1191,7 +1191,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -1299,7 +1299,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>17</v>
       </c>
@@ -1367,12 +1367,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAD555C1-39C7-F145-9423-1631B9A5A54C}">
   <dimension ref="A1:V73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="7"/>
+    <col min="1" max="16384" width="10.85546875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>70</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>154</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H2" s="7">
         <v>950</v>
@@ -1469,20 +1469,20 @@
         <v>41</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K2" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="M2" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="N2" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="L2" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="M2" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="N2" s="9" t="s">
-        <v>161</v>
-      </c>
       <c r="O2" s="10" t="s">
         <v>152</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>71</v>
       </c>
@@ -1528,25 +1528,25 @@
         <v>154</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>41</v>
       </c>
       <c r="J3" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K3" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O3" s="10" t="s">
         <v>152</v>
@@ -1573,7 +1573,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>72</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>154</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H4" s="7">
         <v>975</v>
@@ -1602,19 +1602,19 @@
         <v>41</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L4" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O4" s="10" t="s">
         <v>152</v>
@@ -1641,7 +1641,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>73</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>154</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H5" s="7">
         <v>950</v>
@@ -1670,19 +1670,19 @@
         <v>41</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L5" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M5" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N5" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O5" s="10" t="s">
         <v>152</v>
@@ -1709,7 +1709,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>74</v>
       </c>
@@ -1729,7 +1729,7 @@
         <v>154</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H6" s="7">
         <v>950</v>
@@ -1738,19 +1738,19 @@
         <v>41</v>
       </c>
       <c r="J6" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N6" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O6" s="10" t="s">
         <v>152</v>
@@ -1777,7 +1777,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>75</v>
       </c>
@@ -1797,7 +1797,7 @@
         <v>154</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H7" s="7">
         <v>975</v>
@@ -1806,19 +1806,19 @@
         <v>41</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N7" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>152</v>
@@ -1845,7 +1845,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>76</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>154</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H8" s="7">
         <v>940</v>
@@ -1874,19 +1874,19 @@
         <v>41</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L8" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N8" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O8" s="10" t="s">
         <v>152</v>
@@ -1913,7 +1913,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>77</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>154</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H9" s="7">
         <v>960</v>
@@ -1942,19 +1942,19 @@
         <v>41</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L9" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N9" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O9" s="10" t="s">
         <v>152</v>
@@ -1981,7 +1981,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>78</v>
       </c>
@@ -2001,7 +2001,7 @@
         <v>154</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H10" s="7">
         <v>925</v>
@@ -2010,19 +2010,19 @@
         <v>41</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L10" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M10" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N10" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O10" s="10" t="s">
         <v>152</v>
@@ -2049,7 +2049,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>79</v>
       </c>
@@ -2069,7 +2069,7 @@
         <v>154</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H11" s="7">
         <v>1000</v>
@@ -2078,19 +2078,19 @@
         <v>41</v>
       </c>
       <c r="J11" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L11" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M11" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N11" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O11" s="10" t="s">
         <v>152</v>
@@ -2117,7 +2117,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>80</v>
       </c>
@@ -2137,7 +2137,7 @@
         <v>154</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H12" s="7">
         <v>975</v>
@@ -2146,19 +2146,19 @@
         <v>41</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M12" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N12" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O12" s="10" t="s">
         <v>152</v>
@@ -2185,7 +2185,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>81</v>
       </c>
@@ -2205,7 +2205,7 @@
         <v>154</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H13" s="7">
         <v>950</v>
@@ -2214,19 +2214,19 @@
         <v>41</v>
       </c>
       <c r="J13" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N13" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O13" s="10" t="s">
         <v>152</v>
@@ -2253,7 +2253,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="14" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>82</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>154</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H14" s="7">
         <v>1000</v>
@@ -2282,19 +2282,19 @@
         <v>41</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N14" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O14" s="10" t="s">
         <v>152</v>
@@ -2321,7 +2321,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>83</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>154</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H15" s="7">
         <v>900</v>
@@ -2350,19 +2350,19 @@
         <v>41</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O15" s="10" t="s">
         <v>152</v>
@@ -2389,7 +2389,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="16" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>84</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>154</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H16" s="7">
         <v>925</v>
@@ -2418,19 +2418,19 @@
         <v>41</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K16" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N16" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O16" s="10" t="s">
         <v>152</v>
@@ -2457,7 +2457,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="17" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>85</v>
       </c>
@@ -2477,7 +2477,7 @@
         <v>154</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H17" s="7">
         <v>925</v>
@@ -2486,19 +2486,19 @@
         <v>41</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O17" s="10" t="s">
         <v>152</v>
@@ -2525,7 +2525,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>86</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>154</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H18" s="7">
         <v>950</v>
@@ -2554,19 +2554,19 @@
         <v>41</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K18" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N18" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O18" s="10" t="s">
         <v>152</v>
@@ -2593,7 +2593,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>87</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>154</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H19" s="7">
         <v>950</v>
@@ -2622,19 +2622,19 @@
         <v>41</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L19" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M19" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O19" s="10" t="s">
         <v>152</v>
@@ -2661,7 +2661,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="20" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>88</v>
       </c>
@@ -2681,7 +2681,7 @@
         <v>154</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H20" s="7">
         <v>1010</v>
@@ -2690,19 +2690,19 @@
         <v>41</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K20" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L20" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N20" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O20" s="10" t="s">
         <v>152</v>
@@ -2729,7 +2729,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="21" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>89</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>154</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H21" s="7">
         <v>950</v>
@@ -2758,19 +2758,19 @@
         <v>41</v>
       </c>
       <c r="J21" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L21" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M21" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O21" s="10" t="s">
         <v>152</v>
@@ -2797,7 +2797,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="22" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>90</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>154</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H22" s="7">
         <v>1000</v>
@@ -2826,19 +2826,19 @@
         <v>41</v>
       </c>
       <c r="J22" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L22" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M22" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N22" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O22" s="10" t="s">
         <v>152</v>
@@ -2865,7 +2865,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>91</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>154</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H23" s="7">
         <v>925</v>
@@ -2894,19 +2894,19 @@
         <v>41</v>
       </c>
       <c r="J23" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L23" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M23" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O23" s="10" t="s">
         <v>152</v>
@@ -2933,7 +2933,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="24" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>92</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>154</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H24" s="7">
         <v>900</v>
@@ -2962,19 +2962,19 @@
         <v>41</v>
       </c>
       <c r="J24" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L24" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M24" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N24" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O24" s="10" t="s">
         <v>152</v>
@@ -3001,7 +3001,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="25" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>93</v>
       </c>
@@ -3021,25 +3021,25 @@
         <v>154</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I25" s="7" t="s">
         <v>41</v>
       </c>
       <c r="J25" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K25" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L25" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M25" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O25" s="10" t="s">
         <v>152</v>
@@ -3066,7 +3066,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="26" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>94</v>
       </c>
@@ -3086,7 +3086,7 @@
         <v>154</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H26" s="7">
         <v>975</v>
@@ -3095,19 +3095,19 @@
         <v>41</v>
       </c>
       <c r="J26" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L26" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M26" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N26" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O26" s="10" t="s">
         <v>152</v>
@@ -3134,7 +3134,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="27" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>95</v>
       </c>
@@ -3154,7 +3154,7 @@
         <v>154</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H27" s="7">
         <v>1000</v>
@@ -3163,19 +3163,19 @@
         <v>41</v>
       </c>
       <c r="J27" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K27" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L27" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M27" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>152</v>
@@ -3202,7 +3202,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="28" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>96</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>154</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H28" s="7">
         <v>1000</v>
@@ -3231,19 +3231,19 @@
         <v>41</v>
       </c>
       <c r="J28" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L28" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M28" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N28" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O28" s="10" t="s">
         <v>152</v>
@@ -3270,7 +3270,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="29" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>97</v>
       </c>
@@ -3290,7 +3290,7 @@
         <v>154</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H29" s="7">
         <v>1000</v>
@@ -3299,19 +3299,19 @@
         <v>41</v>
       </c>
       <c r="J29" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K29" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L29" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M29" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O29" s="10" t="s">
         <v>152</v>
@@ -3338,7 +3338,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="30" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>98</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>154</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H30" s="7">
         <v>950</v>
@@ -3367,19 +3367,19 @@
         <v>41</v>
       </c>
       <c r="J30" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L30" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M30" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N30" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O30" s="10" t="s">
         <v>152</v>
@@ -3406,7 +3406,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="31" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>99</v>
       </c>
@@ -3426,7 +3426,7 @@
         <v>154</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H31" s="7">
         <v>950</v>
@@ -3435,19 +3435,19 @@
         <v>41</v>
       </c>
       <c r="J31" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K31" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L31" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M31" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O31" s="10" t="s">
         <v>152</v>
@@ -3474,7 +3474,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="32" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>100</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>154</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H32" s="7">
         <v>950</v>
@@ -3503,19 +3503,19 @@
         <v>41</v>
       </c>
       <c r="J32" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K32" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L32" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M32" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N32" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O32" s="10" t="s">
         <v>152</v>
@@ -3542,7 +3542,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="33" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>101</v>
       </c>
@@ -3562,25 +3562,25 @@
         <v>154</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I33" s="7" t="s">
         <v>41</v>
       </c>
       <c r="J33" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K33" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L33" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M33" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O33" s="10" t="s">
         <v>152</v>
@@ -3607,7 +3607,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="34" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>102</v>
       </c>
@@ -3627,7 +3627,7 @@
         <v>154</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H34" s="7">
         <v>950</v>
@@ -3636,19 +3636,19 @@
         <v>41</v>
       </c>
       <c r="J34" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K34" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L34" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M34" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N34" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O34" s="10" t="s">
         <v>152</v>
@@ -3675,7 +3675,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="35" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>103</v>
       </c>
@@ -3695,7 +3695,7 @@
         <v>154</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H35" s="7">
         <v>1000</v>
@@ -3704,19 +3704,19 @@
         <v>41</v>
       </c>
       <c r="J35" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K35" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L35" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M35" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O35" s="10" t="s">
         <v>152</v>
@@ -3743,7 +3743,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="36" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>104</v>
       </c>
@@ -3763,7 +3763,7 @@
         <v>154</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H36" s="7">
         <v>950</v>
@@ -3772,19 +3772,19 @@
         <v>41</v>
       </c>
       <c r="J36" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K36" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L36" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M36" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N36" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O36" s="10" t="s">
         <v>152</v>
@@ -3811,7 +3811,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="37" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
         <v>105</v>
       </c>
@@ -3831,7 +3831,7 @@
         <v>154</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H37" s="7">
         <v>925</v>
@@ -3840,19 +3840,19 @@
         <v>41</v>
       </c>
       <c r="J37" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K37" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L37" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M37" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O37" s="10" t="s">
         <v>152</v>
@@ -3879,7 +3879,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="38" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
         <v>106</v>
       </c>
@@ -3899,7 +3899,7 @@
         <v>154</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H38" s="7">
         <v>800</v>
@@ -3908,19 +3908,19 @@
         <v>41</v>
       </c>
       <c r="J38" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L38" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M38" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N38" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O38" s="10" t="s">
         <v>152</v>
@@ -3947,7 +3947,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="39" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>107</v>
       </c>
@@ -3967,7 +3967,7 @@
         <v>154</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H39" s="7">
         <v>945</v>
@@ -3976,19 +3976,19 @@
         <v>41</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L39" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M39" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O39" s="10" t="s">
         <v>152</v>
@@ -4015,7 +4015,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="40" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>108</v>
       </c>
@@ -4035,7 +4035,7 @@
         <v>154</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H40" s="7">
         <v>1000</v>
@@ -4044,19 +4044,19 @@
         <v>41</v>
       </c>
       <c r="J40" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K40" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L40" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M40" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N40" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O40" s="10" t="s">
         <v>152</v>
@@ -4083,7 +4083,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="41" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>109</v>
       </c>
@@ -4103,7 +4103,7 @@
         <v>154</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H41" s="7">
         <v>850</v>
@@ -4112,19 +4112,19 @@
         <v>41</v>
       </c>
       <c r="J41" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K41" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L41" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M41" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>152</v>
@@ -4151,7 +4151,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="42" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
         <v>110</v>
       </c>
@@ -4171,7 +4171,7 @@
         <v>154</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H42" s="7">
         <v>1000</v>
@@ -4180,19 +4180,19 @@
         <v>41</v>
       </c>
       <c r="J42" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K42" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L42" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M42" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N42" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O42" s="10" t="s">
         <v>152</v>
@@ -4219,7 +4219,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="43" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>111</v>
       </c>
@@ -4239,7 +4239,7 @@
         <v>154</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H43" s="7">
         <v>950</v>
@@ -4248,19 +4248,19 @@
         <v>41</v>
       </c>
       <c r="J43" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L43" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M43" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O43" s="10" t="s">
         <v>152</v>
@@ -4287,7 +4287,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>112</v>
       </c>
@@ -4307,7 +4307,7 @@
         <v>154</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H44" s="7">
         <v>950</v>
@@ -4316,19 +4316,19 @@
         <v>41</v>
       </c>
       <c r="J44" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K44" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L44" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M44" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N44" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O44" s="10" t="s">
         <v>152</v>
@@ -4355,7 +4355,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>113</v>
       </c>
@@ -4375,7 +4375,7 @@
         <v>154</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H45" s="7">
         <v>1000</v>
@@ -4384,19 +4384,19 @@
         <v>41</v>
       </c>
       <c r="J45" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K45" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L45" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M45" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O45" s="10" t="s">
         <v>152</v>
@@ -4423,7 +4423,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="46" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
         <v>114</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>154</v>
       </c>
       <c r="G46" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H46" s="7">
         <v>1000</v>
@@ -4452,19 +4452,19 @@
         <v>41</v>
       </c>
       <c r="J46" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K46" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L46" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M46" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N46" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O46" s="10" t="s">
         <v>152</v>
@@ -4491,7 +4491,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="47" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>115</v>
       </c>
@@ -4511,7 +4511,7 @@
         <v>154</v>
       </c>
       <c r="G47" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H47" s="7">
         <v>1000</v>
@@ -4520,19 +4520,19 @@
         <v>41</v>
       </c>
       <c r="J47" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K47" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L47" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M47" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O47" s="10" t="s">
         <v>152</v>
@@ -4559,7 +4559,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="48" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>116</v>
       </c>
@@ -4579,7 +4579,7 @@
         <v>154</v>
       </c>
       <c r="G48" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H48" s="7">
         <v>925</v>
@@ -4588,19 +4588,19 @@
         <v>41</v>
       </c>
       <c r="J48" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K48" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L48" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M48" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N48" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O48" s="10" t="s">
         <v>152</v>
@@ -4627,7 +4627,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="49" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>117</v>
       </c>
@@ -4647,7 +4647,7 @@
         <v>154</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H49" s="7">
         <v>1000</v>
@@ -4656,19 +4656,19 @@
         <v>41</v>
       </c>
       <c r="J49" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K49" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L49" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M49" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O49" s="10" t="s">
         <v>152</v>
@@ -4695,7 +4695,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="50" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>118</v>
       </c>
@@ -4715,7 +4715,7 @@
         <v>154</v>
       </c>
       <c r="G50" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H50" s="7">
         <v>1000</v>
@@ -4724,19 +4724,19 @@
         <v>41</v>
       </c>
       <c r="J50" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K50" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L50" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M50" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N50" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O50" s="10" t="s">
         <v>152</v>
@@ -4763,7 +4763,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="51" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>119</v>
       </c>
@@ -4783,7 +4783,7 @@
         <v>154</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H51" s="7">
         <v>1000</v>
@@ -4792,19 +4792,19 @@
         <v>41</v>
       </c>
       <c r="J51" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K51" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L51" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M51" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O51" s="10" t="s">
         <v>152</v>
@@ -4831,7 +4831,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="52" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
         <v>120</v>
       </c>
@@ -4851,25 +4851,25 @@
         <v>154</v>
       </c>
       <c r="G52" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I52" s="7" t="s">
         <v>41</v>
       </c>
       <c r="J52" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K52" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L52" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M52" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N52" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O52" s="10" t="s">
         <v>152</v>
@@ -4896,7 +4896,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="53" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>121</v>
       </c>
@@ -4916,7 +4916,7 @@
         <v>154</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H53" s="7">
         <v>950</v>
@@ -4925,19 +4925,19 @@
         <v>41</v>
       </c>
       <c r="J53" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K53" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L53" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M53" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O53" s="10" t="s">
         <v>152</v>
@@ -4964,7 +4964,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="54" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
         <v>122</v>
       </c>
@@ -4984,7 +4984,7 @@
         <v>154</v>
       </c>
       <c r="G54" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H54" s="7">
         <v>1000</v>
@@ -4993,19 +4993,19 @@
         <v>41</v>
       </c>
       <c r="J54" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K54" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L54" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M54" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N54" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O54" s="10" t="s">
         <v>152</v>
@@ -5032,7 +5032,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="55" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>123</v>
       </c>
@@ -5052,7 +5052,7 @@
         <v>154</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H55" s="7">
         <v>950</v>
@@ -5061,19 +5061,19 @@
         <v>41</v>
       </c>
       <c r="J55" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K55" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L55" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M55" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N55" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O55" s="10" t="s">
         <v>152</v>
@@ -5100,7 +5100,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="56" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
         <v>124</v>
       </c>
@@ -5120,7 +5120,7 @@
         <v>154</v>
       </c>
       <c r="G56" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H56" s="7">
         <v>975</v>
@@ -5129,19 +5129,19 @@
         <v>41</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K56" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L56" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M56" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N56" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O56" s="10" t="s">
         <v>152</v>
@@ -5168,7 +5168,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="57" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>125</v>
       </c>
@@ -5188,7 +5188,7 @@
         <v>154</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H57" s="7">
         <v>1000</v>
@@ -5197,19 +5197,19 @@
         <v>41</v>
       </c>
       <c r="J57" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K57" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L57" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M57" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N57" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O57" s="10" t="s">
         <v>152</v>
@@ -5236,7 +5236,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="58" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
         <v>126</v>
       </c>
@@ -5256,7 +5256,7 @@
         <v>154</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H58" s="7">
         <v>950</v>
@@ -5265,19 +5265,19 @@
         <v>41</v>
       </c>
       <c r="J58" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K58" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L58" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M58" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N58" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O58" s="10" t="s">
         <v>152</v>
@@ -5304,7 +5304,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="59" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>127</v>
       </c>
@@ -5324,7 +5324,7 @@
         <v>154</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H59" s="7">
         <v>950</v>
@@ -5333,19 +5333,19 @@
         <v>41</v>
       </c>
       <c r="J59" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K59" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L59" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M59" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N59" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O59" s="10" t="s">
         <v>152</v>
@@ -5372,7 +5372,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="60" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
         <v>128</v>
       </c>
@@ -5392,7 +5392,7 @@
         <v>154</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H60" s="7">
         <v>1000</v>
@@ -5401,19 +5401,19 @@
         <v>41</v>
       </c>
       <c r="J60" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K60" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L60" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M60" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N60" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O60" s="10" t="s">
         <v>152</v>
@@ -5440,7 +5440,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="61" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
         <v>129</v>
       </c>
@@ -5460,7 +5460,7 @@
         <v>154</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H61" s="7">
         <v>950</v>
@@ -5469,19 +5469,19 @@
         <v>41</v>
       </c>
       <c r="J61" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K61" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L61" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M61" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O61" s="10" t="s">
         <v>152</v>
@@ -5508,7 +5508,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="62" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>130</v>
       </c>
@@ -5528,7 +5528,7 @@
         <v>154</v>
       </c>
       <c r="G62" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H62" s="7">
         <v>950</v>
@@ -5537,19 +5537,19 @@
         <v>41</v>
       </c>
       <c r="J62" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K62" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L62" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M62" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N62" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O62" s="10" t="s">
         <v>152</v>
@@ -5576,7 +5576,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="63" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>131</v>
       </c>
@@ -5596,7 +5596,7 @@
         <v>154</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H63" s="7">
         <v>1000</v>
@@ -5605,19 +5605,19 @@
         <v>41</v>
       </c>
       <c r="J63" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K63" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L63" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M63" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O63" s="10" t="s">
         <v>152</v>
@@ -5644,7 +5644,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="64" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>132</v>
       </c>
@@ -5664,7 +5664,7 @@
         <v>154</v>
       </c>
       <c r="G64" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H64" s="7">
         <v>950</v>
@@ -5673,19 +5673,19 @@
         <v>41</v>
       </c>
       <c r="J64" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K64" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L64" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M64" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N64" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O64" s="10" t="s">
         <v>152</v>
@@ -5712,7 +5712,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="65" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>133</v>
       </c>
@@ -5732,25 +5732,25 @@
         <v>154</v>
       </c>
       <c r="G65" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I65" s="7" t="s">
         <v>41</v>
       </c>
       <c r="J65" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K65" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L65" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M65" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O65" s="10" t="s">
         <v>152</v>
@@ -5777,7 +5777,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="66" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>134</v>
       </c>
@@ -5797,7 +5797,7 @@
         <v>154</v>
       </c>
       <c r="G66" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H66" s="7">
         <v>950</v>
@@ -5806,19 +5806,19 @@
         <v>41</v>
       </c>
       <c r="J66" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K66" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L66" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M66" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N66" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O66" s="10" t="s">
         <v>152</v>
@@ -5845,7 +5845,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="67" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>135</v>
       </c>
@@ -5865,7 +5865,7 @@
         <v>154</v>
       </c>
       <c r="G67" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H67" s="7">
         <v>950</v>
@@ -5874,19 +5874,19 @@
         <v>41</v>
       </c>
       <c r="J67" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K67" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L67" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M67" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O67" s="10" t="s">
         <v>152</v>
@@ -5913,7 +5913,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="68" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>136</v>
       </c>
@@ -5933,7 +5933,7 @@
         <v>154</v>
       </c>
       <c r="G68" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H68" s="7">
         <v>900</v>
@@ -5942,19 +5942,19 @@
         <v>41</v>
       </c>
       <c r="J68" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K68" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L68" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M68" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N68" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O68" s="10" t="s">
         <v>152</v>
@@ -5981,7 +5981,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="69" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>137</v>
       </c>
@@ -6001,7 +6001,7 @@
         <v>154</v>
       </c>
       <c r="G69" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H69" s="7">
         <v>970</v>
@@ -6010,19 +6010,19 @@
         <v>41</v>
       </c>
       <c r="J69" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K69" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L69" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M69" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N69" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O69" s="10" t="s">
         <v>152</v>
@@ -6049,7 +6049,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="70" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>138</v>
       </c>
@@ -6069,7 +6069,7 @@
         <v>154</v>
       </c>
       <c r="G70" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H70" s="7">
         <v>950</v>
@@ -6078,19 +6078,19 @@
         <v>41</v>
       </c>
       <c r="J70" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K70" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L70" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M70" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N70" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O70" s="10" t="s">
         <v>152</v>
@@ -6117,7 +6117,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="71" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>139</v>
       </c>
@@ -6137,25 +6137,25 @@
         <v>154</v>
       </c>
       <c r="G71" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I71" s="7" t="s">
         <v>41</v>
       </c>
       <c r="J71" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K71" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L71" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M71" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N71" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O71" s="10" t="s">
         <v>152</v>
@@ -6182,7 +6182,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="72" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>140</v>
       </c>
@@ -6202,7 +6202,7 @@
         <v>154</v>
       </c>
       <c r="G72" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H72" s="7">
         <v>950</v>
@@ -6211,19 +6211,19 @@
         <v>41</v>
       </c>
       <c r="J72" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K72" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L72" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M72" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N72" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O72" s="10" t="s">
         <v>152</v>
@@ -6250,7 +6250,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="73" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>141</v>
       </c>
@@ -6270,7 +6270,7 @@
         <v>154</v>
       </c>
       <c r="G73" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H73" s="7">
         <v>900</v>
@@ -6279,19 +6279,19 @@
         <v>41</v>
       </c>
       <c r="J73" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K73" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L73" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="M73" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O73" s="10" t="s">
         <v>152</v>

</xml_diff>